<commit_message>
Add priority to example_specifications.xlsx
</commit_message>
<xml_diff>
--- a/packages/excel-parser/examples/example_specifications.xlsx
+++ b/packages/excel-parser/examples/example_specifications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael.houston/nhs-notify/nhs-notify-supplier-config/packages/event-builder/examples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael.houston/nhs-notify/nhs-notify-supplier-config/packages/excel-parser/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598A88ED-9F51-734C-B42E-480FDDE54AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23582231-933C-B240-9206-1EB3E29C43E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3840" yWindow="-31780" windowWidth="38400" windowHeight="31780" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="800" windowWidth="41120" windowHeight="25780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PackSpecification" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="131">
   <si>
     <t>id</t>
   </si>
@@ -415,6 +415,9 @@
   </si>
   <si>
     <t>approval</t>
+  </si>
+  <si>
+    <t>priority</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1329,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
@@ -1334,16 +1337,18 @@
     <col min="3" max="3" width="38.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.83203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="33.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.33203125" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="32.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="33.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1363,28 +1368,31 @@
         <v>29</v>
       </c>
       <c r="G1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>30</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>31</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>13</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -1403,20 +1411,23 @@
       <c r="F2" t="s">
         <v>43</v>
       </c>
-      <c r="G2" t="s">
-        <v>128</v>
-      </c>
-      <c r="J2">
+      <c r="G2">
+        <v>50</v>
+      </c>
+      <c r="H2" t="s">
+        <v>128</v>
+      </c>
+      <c r="K2">
         <v>20</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>3</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -1435,20 +1446,23 @@
       <c r="F3" t="s">
         <v>48</v>
       </c>
-      <c r="G3" t="s">
-        <v>128</v>
-      </c>
-      <c r="J3">
+      <c r="G3">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>128</v>
+      </c>
+      <c r="K3">
         <v>5</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>3</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1467,20 +1481,23 @@
       <c r="F4" t="s">
         <v>43</v>
       </c>
-      <c r="G4" t="s">
-        <v>128</v>
-      </c>
-      <c r="J4">
+      <c r="G4">
+        <v>50</v>
+      </c>
+      <c r="H4" t="s">
+        <v>128</v>
+      </c>
+      <c r="K4">
         <v>5</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>2</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1499,20 +1516,23 @@
       <c r="F5" t="s">
         <v>56</v>
       </c>
-      <c r="G5" t="s">
-        <v>128</v>
-      </c>
-      <c r="J5">
+      <c r="G5">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>128</v>
+      </c>
+      <c r="K5">
         <v>5</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>1</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>57</v>
       </c>
@@ -1531,29 +1551,32 @@
       <c r="F6" t="s">
         <v>43</v>
       </c>
-      <c r="G6" t="s">
-        <v>128</v>
+      <c r="G6">
+        <v>20</v>
       </c>
       <c r="H6" t="s">
+        <v>128</v>
+      </c>
+      <c r="I6" t="s">
         <v>60</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>61</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>4</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>3</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>50</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 E1:M1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1 H1:N1 E1:F1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>